<commit_message>
Add unread guidance notifications with DB-backed badge system
</commit_message>
<xml_diff>
--- a/case_register.xlsx
+++ b/case_register.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P28"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -445,24 +445,1405 @@
         <v>Description</v>
       </c>
       <c r="J1" t="str">
+        <v>Date of Case</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Employment Status</v>
+      </c>
+      <c r="L1" t="str">
         <v>Assistance</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Status</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Contacts</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Created By</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>Last Edited By</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>G-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Mr Moretlwa Kerahela</v>
+      </c>
+      <c r="C2" t="str">
+        <v>852216304</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Qabo</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K2" t="str" xml:space="preserve">
+        <v xml:space="preserve">He won a tender from Huiku Trust and then in three days the tender got terminated, so he is requesting for compensation of damage attempted prior to contract termination. Mr Moretlwa came to the Gantsi office complaining that Huiku Trust failed to pay him after terminating his contract to clear along roads. The contract was terminated 3 days after being issued. Mr Moretlwa requested a written letter of the termination but it was not issued. He said all he is requesting for the expenses’ summing up to P15731.00 +P300.00 which was spent on transport or taxi fees. The client also showed that he has been to BONELA where, the Huiku trust agreed to pay him but they never did.
+The client requested assistance from DITSHWANELO,he wants Huiku to pay him.</v>
+      </c>
+      <c r="L2" t="str" xml:space="preserve">
+        <v xml:space="preserve">We have written letter to both parties to engage them in talks.
+Currently the DITSHWANELO office has requested to meet with the Huiku board but as of today (28/11/2025) they are not available due to the ongoing 6day full council. DITSHWANELO Gantsi office has supporting documents and letters for any further inquiries. We assume they will respond week so we could meet before our closing dates for festive holidays.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N2" t="str">
+        <v>73068392</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>G-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Mr Keofetlhetse Gaeatiwe</v>
+      </c>
+      <c r="C3" t="str">
+        <v>036913294</v>
+      </c>
+      <c r="D3" t="str">
+        <v>1978-06-03</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Khurakhura Ward</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Mrs. Elinah Maseane, who hired Mr. Keofetlhetse's son Xukuri Mothibi Moretlwa, failed to pay him his September 2025 salary. After the office engaged them in negotiations, she was able to pay him severance and the September salary.</v>
+      </c>
+      <c r="L3" t="str">
+        <v>We engaged both parties together in talks and defendant managed to pay complainant P1500.00</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="N3" t="str">
+        <v>75225607/76924010</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>G-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Ms Moipoledi Gabobogwe</v>
+      </c>
+      <c r="C4" t="str">
+        <v>503223720</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Morama</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Other</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Ms Moipoledi Gabobogwe of ID no. 503223720, contact 74892544, came to the office requesting assistance requiring  her boyfriend Mr Oduetse Kabelo of contact 77345790 who she claims infected her the HIV /AIDS intentionally since he alresdy knew his status but choice not to tell her hence having unprotected sex with her for the period of 1year 6months.Ms Moipoledi Gabobogwe found out about the virus through a phone call from an unknown lady claiming to be his babys mother. Together Ms Gabobogwe and Mr Kabelo went to the clinic where it was confirmed that they are positive and he refused to take counselling.</v>
+      </c>
+      <c r="L4" t="str">
+        <v>The case was referred to Bonela as the office would not offer better support than Bonela whom are focused to such cases</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="N4" t="str">
+        <v>74892544</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>G-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Mr Bashi Gobuamang</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Qabo</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Gobuamang Bashi  was posted at Xade by the Department of Wildlife from 2019-2012 and was requested to be transferred to Ngoma Wildlife camp which is based at Kasane. He verbal negotiated refusing to be transferred because he was ill. The issue took turn for the worse when letters of miscoduct were issued to him and he was called for disciplinary hearing. During the hearing his supervisers were bias.By year 02/09/15 the office of the ministry wrote to him for Mitigation and he was Dismissed from public service on the 31/12/2015. During all that time he was not getting any salary.
+Mr Gobuamang wants the salary owned.</v>
+      </c>
+      <c r="L5" t="str">
+        <v>The DITSHWANELO Gantsi Office is looking forward to writing a letter in which both parties may meet and discuss the issue at hand.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>G-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Ms Cgose Kemoneilwe</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>1988-09-20</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Ghanzi</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Bosele Ward</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Family Matter</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Ms Cgose Kemoneilwe complained that she is having conflicts with her husband. She explained that he is physically abusing her and he is cheating with a known person whom is their neighbour. My client would like the office to help her by calling a meeting with both parties as she wants the man to choose who he really wants to be with and also explain how he is going to support their two children.</v>
+      </c>
+      <c r="L6" t="str" xml:space="preserve">
+        <v xml:space="preserve">We managed to meet with both parties they agreed not to separate but rather forgive each other and take care of their children together.
+case was closed after following up after the mediation session.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="N6" t="str">
+        <v>75392303</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>G-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Mr Kegopotswe Sarwanyane</v>
+      </c>
+      <c r="C7" t="str">
+        <v>286311200</v>
+      </c>
+      <c r="D7" t="str">
+        <v>1975-06-15</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Ghanzi</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Kgaphamadi</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Family Matter</v>
+      </c>
+      <c r="K7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Serwanyane complained that his mother did not repay the damages he lost when helping develop his mother's residential plot which was later sold. The damages include connecting electricity, water and building 2 rooms which he built together with his late sister. He requested to be assisted in claiming the losses. He failed to produce any proof of the claims and has no contacts for the people he is complaining about.
+He requested that the office help him by calling his mother to come and pay him what they owe him.</v>
+      </c>
+      <c r="L7" t="str" xml:space="preserve">
+        <v xml:space="preserve">We listened and advised him to look for any individual who may  stand as his witness and the office advised that he should ask the police to company him the known relatives because the office does not have the means to look for his family.
+unproved word on the streets is that he went to prison after almost killing his mother and her mother is under witness protection but it is just a rummer.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N7" t="str">
+        <v>72115802</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>G-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Ms Quba Tshota</v>
+      </c>
+      <c r="C8" t="str">
+        <v>096522803</v>
+      </c>
+      <c r="D8" t="str">
+        <v>1980-01-30</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Qabo</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Qabo</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Civil</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Dispute between two business partners regarding business equipment, more especially a rental tent. Ms Tshota Quba complained to the social worker stationed at Qabo (Miss Tidimalo). Her business partner Ms Texgao Xao misused company money and took the tent. Ms Texgao is now refusing to let her business partner use it.</v>
+      </c>
+      <c r="L8" t="str">
+        <v>requested a meeting with the social worker and Kgosi from the Qabo settlement</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N8" t="str">
+        <v>73918214</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>G-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Ms Lorato Motshabi</v>
+      </c>
+      <c r="C9" t="str">
+        <v>466927610</v>
+      </c>
+      <c r="D9" t="str">
+        <v>1991-07-19</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Moherero</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Molapo</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Ms Motshabi complained that they were not paid by Mr Ditshwene of Keseede Guest House their salaries from November to January. The office called him and he explained that the business had not been doing well, but he managed to get a loan and paid them the same day.</v>
+      </c>
+      <c r="L9" t="str">
+        <v>She was paid the full amount.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="N9" t="str">
+        <v>72874869</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>G-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Mr Tsaa Xuka</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>2002-09-04</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Molapo</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K10" t="str">
+        <v>The client complained that he was not happy about how he was assisted at the Labour office and requested to be accompanied. He was requesting 8 years severance which he claimed Mr Du Plessis owed him.</v>
+      </c>
+      <c r="L10" t="str">
+        <v>The office went to labour offices and meet with a mediation officer and Mr Du Plessis managed to pay the client amounted owed and severance.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="N10" t="str">
+        <v>75239734</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>G-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Mr Dabe Khanxlae</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Bosele</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Mr Dabe explained that Mr Setima took them as a group to his farm to fence the field and clear the bush, but upon finishing he failed to pay them. They came as a group requesting help. The office called Mr Setima and he explained he failed to pay due to the closing of the cattle market from foot and mouth prevention measures, but promised to pay as soon as the market opens. He owes P1500 each to 3 workers who fenced, and P1500 each to those who cleared the field.</v>
+      </c>
+      <c r="L11" t="str">
+        <v>The office once got hold of Mr Setima and he promised to but but has not paid yet. Mr Setima is currently avoiding answering the phone.</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>G-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Mr Ditlhapang Mpopona</v>
+      </c>
+      <c r="C12" t="str">
+        <v>658811300</v>
+      </c>
+      <c r="D12" t="str">
+        <v>1969-01-01</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>Grootlaagte</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Grootlaagte</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Family Matter</v>
+      </c>
+      <c r="K12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Mpopona Ditlhabang complained that his brother Cosmos Soke is trying to still his borehole by making him sign papers tranfer it to his names.
+The issue started after the brothers fought and Mpopona wa arrested and his brother was blackmailed him saying that for him to drop charges is for him to sign the papers.</v>
+      </c>
+      <c r="L12" t="str">
+        <v>The client said he will bring supporting documents but never returned.</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="N12" t="str">
+        <v>73877788</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>G-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Benjamin Tjienda</v>
+      </c>
+      <c r="C13" t="str">
+        <v>280215606</v>
+      </c>
+      <c r="D13" t="str">
+        <v>1974-12-12</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Moherero</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Bosele Ward</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N13" t="str">
+        <v>76525561</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>G-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Daokane Gokailwemang</v>
+      </c>
+      <c r="C14" t="str">
+        <v>677714703</v>
+      </c>
+      <c r="D14" t="str">
+        <v>1976-01-01</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>Ghanzi</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Morama Ward</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Family Matter</v>
+      </c>
+      <c r="K14" t="str" xml:space="preserve">
+        <v xml:space="preserve">He wants his ex girlfriends boyfriend to leave him alone as the boyfriend is harrassing him saying that he almost burnt his house twice. 
+He explained that he reported but the issue has not stopped.</v>
+      </c>
+      <c r="L14" t="str">
+        <v>We tried calling the acussed but failed to reach him or the ex girlfriend.</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N14" t="str">
+        <v>74320215</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>G-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Lepang Lesheto</v>
+      </c>
+      <c r="C15" t="str">
+        <v>405014618</v>
+      </c>
+      <c r="D15" t="str">
+        <v>1984-04-03</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>New Xade</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Meriting Ward</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K15" t="str">
+        <v>He requested that the office assist him as he was transfered from New Xade to Gantsi senior secondary school and they failed to provide accomodation.</v>
+      </c>
+      <c r="L15" t="str">
+        <v>The office have proposed a meeting with the school management.</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N15" t="str">
+        <v>77592718</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>G-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tshekoemang Tlhobolo</v>
+      </c>
+      <c r="C16" t="str">
+        <v>063417204</v>
+      </c>
+      <c r="D16" t="str">
+        <v>1969-12-23</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>Kuke</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Kuke</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Land Dispute</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Mr Tlhobolo Tshekoemang  come to the office requesting that the office help  him claim his late grandfathers farm, he explained that the white man came and found his grandparents settling at a place they called Kobe.</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N16" t="str">
+        <v>72860105</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>G-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Pouveni Mokgatlanyane</v>
+      </c>
+      <c r="C17" t="str">
+        <v>558811301</v>
+      </c>
+      <c r="D17" t="str">
+        <v>1964-02-01</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Moherero</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Kgapamadi</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Land Dispute</v>
+      </c>
+      <c r="K17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Pouveni  Mokgatlanyane presented many issues before the DITSHWANELO Gantsi office those cases are as follow;
+Request for intervention regarding hit and run case in which his uncle Sasane Times Modisapitse was hit and run by a vehicle while walking on the 7th August 1998 by Bashi Balopi but the case never went to court. Apperently the driver never stopped after hitting the uncle and the accussed stayed in hiding for 3days. The client stated that he appealed to the office of the president twice but never got assisted.
+Request for his mother's ploughing field certificate. The client is requesting to be issued a certificate of a ploughing field in Gantsi, at Khurakhura ward , and he has a letter from the court president confirming his claims.
+Residential Plot Quiry-Mr Mokgatlanyane also explained that he applied for a plot at Gaborone in 1991, and in 2001 the ministry of Lands wrote to him offering him a plot at Francistown instead of Gaborone. He explained that he was number 30 but after 30 years he was offered elsewhere by the office trying to hide their corruption practices. Adding to his distress the client also shared that in Gantsi he applied in 1982,1984 and 1989 and still got nothing, that is when he went and applied at Gaborone in 1991.
+Employment - Mr Mokgatlanyane Pouveni also worked at the department of forestry and range resources for 27 years in one scale of B4 having the experience but no promotion.
+Appeal against surcharge involving government vehicle- the client explained that he had an accident with a government truck whilst on duty, but the department surcharged him the whole amount of P76380.60 for maintaining the vehicle instead of cost sharing as it is the case. He also stated that they are still following me with surcharge.
+Mr Pouveni Mokgatlanyane  requested that he really needs to be assisted to get back his original plot in Gaborone no matter who developed it. Thats his priority as of now and he also requested that he gets assisted as soon as possible.</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Ongoing as the office has wrote to DITSHWANELO headquaters at Gaborone requesting Ms Florah Kedibonye to came and assist with a way forward regarding all the cases presented by the client.</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N17" t="str">
+        <v>72619303</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>G-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Tshetlhane Dintwa</v>
+      </c>
+      <c r="C18" t="str">
+        <v>019816804</v>
+      </c>
+      <c r="D18" t="str">
+        <v>1947-01-01</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Khurakhura Ward</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Land Dispute</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Mr Tshetlhane Dintwa came to the office requesting assistance as his nephwe mr Pragar Tshetlhane has sold his residental plot without his concent . Mr Tshetlhane provided the office with a copy of the plots certificate.</v>
+      </c>
+      <c r="L18" t="str" xml:space="preserve">
+        <v xml:space="preserve">The office managed to contact Mr Pragar Tshetlhane who refused to come to the office.
+The office went to Self Help Housing Agency (SHHA) office where the officer explained that Mr Tshetlhane Dintwa has 2 plots and  1 is transferred to the accused mr Tshetlhane</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N18" t="str">
+        <v>74405383</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>G-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Moronko Dithapelo</v>
+      </c>
+      <c r="C19" t="str">
+        <v>615417904</v>
+      </c>
+      <c r="D19" t="str">
+        <v>1963-01-18</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>Sehitwa</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Kabakae Ward</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Civil</v>
+      </c>
+      <c r="K19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Moronko Dithapelo complained that the Morama Vdc destroyed his property and they are failing to refund and or make  the bricks they destroyed. He explained that they cut some tree branches on the other side of the road and threw the branches into his yard as ordered by the Vdc chairman. The branches destroyed the newly made bricks hence making mr Moronko loss his investment. 
+The client also explained that he went to the Morama ward, Kgosi Molehele. The client was not pleased with the judgement of the kgosi. Apparently the accused refused to coorporate or come for the meeting.</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Ongoing as we requested a meeting with the morama Vdc and the Kgosi</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N19" t="str">
+        <v>77964522</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>G-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Ms Minah Jackane</v>
+      </c>
+      <c r="C20" t="str">
+        <v>317324616</v>
+      </c>
+      <c r="D20" t="str">
+        <v>1984-07-04</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>Ghanzi</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Bosele</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Family Matter</v>
+      </c>
+      <c r="K20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Ms Minah Jackane came to the office and request assistance with a father who is failing to support his two children. She explained that he is working at SR cleaning company. Ms Minah Jackane also said she was given P100.00 only for the month of Febrary .She also explained that one of the children is at a boarding school and usually need some stuff regularly  because other students steal from young ones.
+In other issues she stated that she was left to care for two young children whom their mother had neglected.</v>
+      </c>
+      <c r="L20" t="str" xml:space="preserve">
+        <v xml:space="preserve">The office advised her to report to court and she did . At court it was showed that she once reported and withdraw the case which they explicitly stated that she needs to write a letter to request that her case be reinstained.
+The case was closed as well as the office prepared a mediation in which both parties
+came and the issues were discussed. The mother of the neglected  child agreed to stay with Minah Jackane whom was left with the children without assistance. The mother explained that she was homeless and unemployed but culd move in with Minah Jackane to a stable home where she will help take care of her home.
+The discussions ended with both parties agreeing to the agreements and both parents of the children agreed that they are no longer together so non of them should bother each other.</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N20" t="str">
+        <v>72220184</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P20" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>G-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Mr Kashe Quebi</v>
+      </c>
+      <c r="C21" t="str">
+        <v>119610108</v>
+      </c>
+      <c r="D21" t="str">
+        <v>1967-02-03</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>East Hanahai</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v>Civil</v>
+      </c>
+      <c r="K21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Kashe  Quebi was brutally beaten by a group of man from  Matlo a Rona Rotlhe. Mr Kaashe Quebi and Mr Russia Kodie of ID number 657012809 was also beaten and sustained injuries by the same group as they were suspected to have stolen a cow. Mr Kashe Quebi has also sustained serious injuries as he explained that he is now using tubes to urinate.
+They went to the police superintended 3 times where they were not assisted.</v>
+      </c>
+      <c r="L21" t="str">
+        <v>The office will write to the Police department or superintended.</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N21" t="str">
+        <v>78323660</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P21" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>G-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Dikotane Komiti</v>
+      </c>
+      <c r="C22" t="str">
+        <v>394010208</v>
+      </c>
+      <c r="D22" t="str">
+        <v>1978-01-01</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Mokalagadi</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>Unemployed</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Ncojane</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Bosele</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Land Dispute</v>
+      </c>
+      <c r="K22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mr Dikoloti came to the office with his brothers Emmanuel Dikotane and Kotsi Dikotane seeking assistance regardinga borehole in which their grandfather Mr Dikotane Dikotane gave or went into an agreement with Mr Dineal Mothibi, Modise Dikotane and Mochanako Jackie who offered in the year 2007 to drill the water. In 2007, Mr Dikotane Dikotane requested that they pay rent of P4000.00 per year. They tried to change the name of the syndicate from Dikotane Dikotane to Mokaleng.
+The Dikotanes want other partners to leave their grandparents borehole or pay rent starting from 2007.</v>
+      </c>
+      <c r="L22" t="str">
+        <v>The office have been trying to reach other parties but have not reached any.</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N22" t="str">
+        <v>77307906</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P22" t="str">
+        <v>William Tuahuku</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>G-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Mr Emmaual Dikotane</v>
+      </c>
+      <c r="C23" t="str">
+        <v>184419206</v>
+      </c>
+      <c r="D23" t="str">
+        <v>1980-04-20</v>
+      </c>
+      <c r="E23" t="str">
+        <v>mokgalagadi</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2025-09-25</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Unemployed</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Gantsi</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Bosele</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Land Dispute</v>
+      </c>
+      <c r="K23" t="str">
+        <v>The client was complaining that the Charleshill District Council denied him an opportunity inwhich he was denied to attend aninterview.</v>
+      </c>
+      <c r="L23" t="str">
+        <v>case closed as his request was unsuccessful.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Closed</v>
+      </c>
+      <c r="N23" t="str">
+        <v>73558365</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P23" t="str">
+        <v>William Tuahuku</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>G-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Mr Pula Isanang</v>
+      </c>
+      <c r="C24" t="str">
+        <v>409817607</v>
+      </c>
+      <c r="D24" t="str">
+        <v>1972-01-01</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Mokgalagadi</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>kgaphamadi</v>
+      </c>
+      <c r="I24" t="str">
+        <v>kgaphamadi</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Land Dispute</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Mr Pula Isanang explained that he bought a borehole from the government at Water Affairs in 2014 at a price of P20000 (twenty thousand pula) and later paid the retal arrears of P16 150.70 with the hope that in future he could own the borehole since the water right holder (Kerebe Syndicate) gave a written consent that the borehole be registered in his names prior to a convenant he made with this particular syndicate- to buy the borehole . Prior to this convenant, Kerebe Syndicate owed DWA in lease arrears amounting to P16 150.70.</v>
+      </c>
+      <c r="L24" t="str" xml:space="preserve">
+        <v xml:space="preserve">We asked about at the office at Water Affairs but were told that the right person with all the information is at leave and will be available June.
+I also needed advice from my supervisers as i do not know that the government sold boreholes.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N24" t="str">
+        <v>72141675</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P24" t="str">
+        <v>William Tuahuku</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>G-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Ms Keletso Pearl Gaborakanelwe</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v>1986-03-21</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Ms Keletso Pearl Gaborakanelwe come and reported that she was hired at the mine in Gantsi under the company AMS at the Motheo Copper Mine, was driving trucks started in August 2022 and in the same month of August she was (diagonosed) with Fibroids condition. The Dr advised with the medical report that they decrease her working hours report was delayed after sometimes of her not being well everytime she drives a truck always (bleeding heavely) without her consent they suggested that she has to do operation (removing fibroids) and she was moved from one pit to the other (new one).December 2025 she was still not well. She was given off days. All the incidents she was always reporting them up until one day when she was on a night shift, when she was about to start a truck she heard a lot of noise when she checked   only to find out that the stairs where the truck passes were remained and her boss was besidesthe truck, she just corrected the stairs and went back to do her usual job and she was fired for that.
+The client has shown issues of unfair treatmet at work and unfair dismissial.
+She is requesting justice.</v>
+      </c>
+      <c r="L25" t="str">
+        <v>The office has wrote to AMS mine and got a respond to attend investigation interview. The interview was done and the company said they will get back to us.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P25" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>G-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Ms Tjiwneno Mokgatlanyane</v>
+      </c>
+      <c r="C26" t="str">
+        <v>909827702</v>
+      </c>
+      <c r="D26" t="str">
+        <v>1962-01-18</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Moherero</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v>Ghanzi</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Kgaphamadi south ward</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Inheritence Despute</v>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N26" t="str">
+        <v>75825286</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P26" t="str">
+        <v>William Tuahuku</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>G-026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Mr Phemelo</v>
+      </c>
+      <c r="C27" t="str">
+        <v>383515104</v>
+      </c>
+      <c r="D27" t="str">
+        <v>1978-01-07</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Mokalaka</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v>Francistown</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v>Labour Dispute</v>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N27" t="str">
+        <v>74488660</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>G-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Ms Qose Dabe</v>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v>1989-01-30</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Mosarwa</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v>Ghanzi</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Bosele Ward</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Family Matter</v>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N28" t="str">
+        <v>72359992</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Kaku Bafedile</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Kaku Bafedile</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -484,7 +1865,7 @@
         <v>Total</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +1873,7 @@
         <v>Ongoing</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -500,7 +1881,7 @@
         <v>Pending</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -508,7 +1889,7 @@
         <v>Closed</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>